<commit_message>
Ejercicio tabla 2 fixed
</commit_message>
<xml_diff>
--- a/Ejercicios Normalizacion/Ejercicio 2.xlsx
+++ b/Ejercicios Normalizacion/Ejercicio 2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\lyfter\Ejercicios Modulo Python\DUAD\Ejercicios Normalizacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10070F0-B4AF-46A6-B65C-67FBE54ED04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38184A14-D0F2-4955-9634-B25EFC28BB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{7351F4FB-C425-406A-B187-042F913AE7DA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="51">
   <si>
     <t>VIN</t>
   </si>
@@ -164,9 +164,6 @@
     <t>id</t>
   </si>
   <si>
-    <t>Model Year</t>
-  </si>
-  <si>
     <t>Id</t>
   </si>
   <si>
@@ -176,7 +173,25 @@
     <t>Cars_owners</t>
   </si>
   <si>
-    <t>Insurance</t>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>InsuranceCompanies</t>
+  </si>
+  <si>
+    <t>CompanyName</t>
+  </si>
+  <si>
+    <t>InsuranceId</t>
+  </si>
+  <si>
+    <t>Cars_Insurance</t>
+  </si>
+  <si>
+    <t>CarInfo</t>
+  </si>
+  <si>
+    <t>CarInfoID</t>
   </si>
 </sst>
 </file>
@@ -579,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0A58B94-95FB-4544-AD2B-67FDB9BA65D1}">
-  <dimension ref="A2:N28"/>
+  <dimension ref="A2:N39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.85546875" customWidth="1"/>
@@ -588,9 +603,10 @@
     <col min="6" max="6" width="13.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.140625" customWidth="1"/>
     <col min="8" max="8" width="12.28515625" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="18.5703125" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" customWidth="1"/>
     <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="12" max="12" width="19.28515625" customWidth="1"/>
     <col min="13" max="13" width="18.28515625" customWidth="1"/>
     <col min="14" max="14" width="15.42578125" customWidth="1"/>
   </cols>
@@ -770,27 +786,21 @@
         <v>37</v>
       </c>
       <c r="K15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>0</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G16" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="L16" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>39</v>
@@ -806,14 +816,8 @@
       <c r="E17" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>18</v>
+      <c r="F17" s="1">
+        <v>1</v>
       </c>
       <c r="L17" s="1">
         <v>1</v>
@@ -832,14 +836,8 @@
       <c r="E18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>19</v>
+      <c r="F18" s="1">
+        <v>2</v>
       </c>
       <c r="L18" s="1">
         <v>2</v>
@@ -858,14 +856,8 @@
       <c r="E19" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>20</v>
+      <c r="F19" s="1">
+        <v>3</v>
       </c>
       <c r="L19" s="1">
         <v>3</v>
@@ -890,12 +882,12 @@
     </row>
     <row r="22" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="3:14" x14ac:dyDescent="0.25">
       <c r="D23" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>6</v>
@@ -903,7 +895,7 @@
       <c r="F23" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J23" t="s">
+      <c r="I23" t="s">
         <v>45</v>
       </c>
     </row>
@@ -917,16 +909,13 @@
       <c r="F24" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="J24" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="K24" s="1" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="N24" s="1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -940,16 +929,13 @@
       <c r="F25" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="K25" s="1">
-        <v>1</v>
-      </c>
-      <c r="L25" s="1">
-        <v>1</v>
-      </c>
-      <c r="M25" s="1" t="s">
+      <c r="J25" s="1">
+        <v>1</v>
+      </c>
+      <c r="K25" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N25" s="1" t="s">
+      <c r="L25" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -963,16 +949,13 @@
       <c r="F26" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="K26" s="1">
-        <v>2</v>
-      </c>
-      <c r="L26" s="1">
-        <v>2</v>
-      </c>
-      <c r="M26" s="1" t="s">
+      <c r="J26" s="1">
+        <v>2</v>
+      </c>
+      <c r="K26" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N26" s="1" t="s">
+      <c r="L26" s="1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -986,31 +969,155 @@
       <c r="F27" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K27" s="1">
-        <v>3</v>
-      </c>
-      <c r="L27" s="1">
-        <v>3</v>
-      </c>
-      <c r="M27" s="1" t="s">
+      <c r="J27" s="1">
+        <v>3</v>
+      </c>
+      <c r="K27" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N27" s="1" t="s">
+      <c r="L27" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="28" spans="3:14" x14ac:dyDescent="0.25">
-      <c r="K28" s="1">
+      <c r="J28" s="1">
         <v>4</v>
       </c>
-      <c r="L28" s="1">
+      <c r="K28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="30" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="D31" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H31" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="M28" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="N28" s="1" t="s">
-        <v>36</v>
+      <c r="J31" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="32" spans="3:14" x14ac:dyDescent="0.25">
+      <c r="D32" s="1">
+        <v>1</v>
+      </c>
+      <c r="E32" s="1">
+        <v>2003</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L32" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M32" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D33" s="1">
+        <v>2</v>
+      </c>
+      <c r="E33" s="1">
+        <v>2014</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K33" s="1">
+        <v>1</v>
+      </c>
+      <c r="L33" s="1">
+        <v>1</v>
+      </c>
+      <c r="M33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D34" s="1">
+        <v>3</v>
+      </c>
+      <c r="E34" s="1">
+        <v>2015</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K34" s="1">
+        <v>2</v>
+      </c>
+      <c r="L34" s="1">
+        <v>1</v>
+      </c>
+      <c r="M34" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="K35" s="1">
+        <v>3</v>
+      </c>
+      <c r="L35" s="1">
+        <v>2</v>
+      </c>
+      <c r="M35" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="K36" s="1">
+        <v>4</v>
+      </c>
+      <c r="L36" s="1">
+        <v>3</v>
+      </c>
+      <c r="M36" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="G39" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>